<commit_message>
Add foreign bank charges to receipts & payments
Model bank fees deducted on foreign remittances (e.g. party transfers
USD 10,000, bank deducts USD 100, USD 9,900 received) as a separate expense:

- FC Amount (Gross) settles the invoice and drives forex gain/(loss)
- Foreign Bank Charges (FC) is a new input column, booked separately
- Net Bank Movement (FC/Base) shows what actually hit the bank
  (receipts = gross - charges; payments = gross + charges)
- Dashboard totals foreign bank charges and net cash separately so the
  forex figure stays clean; Read Me documents the treatment

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Mkxh7BaYytzCHatgymYrfu
</commit_message>
<xml_diff>
--- a/Foreign_Gain_Loss_Workbook.xlsx
+++ b/Foreign_Gain_Loss_Workbook.xlsx
@@ -25,11 +25,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="dd-mmm-yyyy"/>
     <numFmt numFmtId="166" formatCode="0.0000"/>
-    <numFmt numFmtId="167" formatCode="#,##0.00;[Red](#,##0.00)"/>
+    <numFmt numFmtId="167" formatCode="#,##0.00;(#,##0.00)"/>
+    <numFmt numFmtId="168" formatCode="#,##0.00;[Red](#,##0.00)"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -192,7 +193,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -259,7 +260,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -273,6 +274,9 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="167" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
@@ -436,21 +440,25 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="tblSettlements" displayName="tblSettlements" ref="A4:L12" headerRowCount="1">
-  <autoFilter ref="A4:L12"/>
-  <tableColumns count="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="tblSettlements" displayName="tblSettlements" ref="A4:P12" headerRowCount="1">
+  <autoFilter ref="A4:P12"/>
+  <tableColumns count="16">
     <tableColumn id="1" name="Settlement Ref"/>
     <tableColumn id="2" name="Settlement Type"/>
     <tableColumn id="3" name="Party Name"/>
     <tableColumn id="4" name="Currency"/>
     <tableColumn id="5" name="Settlement Date"/>
-    <tableColumn id="6" name="FC Amount"/>
+    <tableColumn id="6" name="FC Amount (Gross)"/>
     <tableColumn id="7" name="Settlement Rate"/>
-    <tableColumn id="8" name="Settlement Value (Base)"/>
-    <tableColumn id="9" name="FC Allocated"/>
-    <tableColumn id="10" name="FC Unallocated"/>
-    <tableColumn id="11" name="Allocation Status"/>
-    <tableColumn id="12" name="Narration"/>
+    <tableColumn id="8" name="Foreign Bank Charges (FC)"/>
+    <tableColumn id="9" name="Net Bank Movement (FC)"/>
+    <tableColumn id="10" name="Settlement Value (Base)"/>
+    <tableColumn id="11" name="Bank Charges (Base)"/>
+    <tableColumn id="12" name="Net Bank Movement (Base)"/>
+    <tableColumn id="13" name="FC Allocated"/>
+    <tableColumn id="14" name="FC Unallocated"/>
+    <tableColumn id="15" name="Allocation Status"/>
+    <tableColumn id="16" name="Narration"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium6" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -775,7 +783,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H32"/>
+  <dimension ref="A1:H39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -943,59 +951,104 @@
       </c>
     </row>
     <row r="27" ht="20" customHeight="1">
-      <c r="A27" s="7" t="inlineStr">
-        <is>
-          <t>CONVENTIONS</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="15" customHeight="1">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>FOREIGN BANK CHARGES</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="28" customHeight="1">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>•  Rate = units of base currency per 1 unit of foreign currency (e.g. INR per 1 USD).</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="15" customHeight="1">
+          <t>When a bank deducts a fee on a foreign remittance (e.g. the party transfers USD 10,000 but only USD 9,900 reaches you, USD 100 taken by the bank):</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="28" customHeight="1">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>•  Blue headers = your input.   Grey headers = automatically calculated, do not overtype.</t>
+          <t>•  Enter the FULL amount transferred in 'FC Amount (Gross)'  →  this settles the invoice and drives the forex gain/(loss).</t>
         </is>
       </c>
     </row>
     <row r="30" ht="28" customHeight="1">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>•  Tables auto-extend: start typing on the row below a table and the formatting &amp; formulas copy down.</t>
+          <t>•  Enter the fee in 'Foreign Bank Charges (FC)'  →  it is booked as a SEPARATE expense, never mixed into forex gain/(loss).</t>
         </is>
       </c>
     </row>
     <row r="31" ht="28" customHeight="1">
       <c r="A31" s="4" t="inlineStr">
         <is>
+          <t>•  'Net Bank Movement' then shows what actually hit your bank (receipts = gross − charges; payments = gross + charges).</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="15" customHeight="1">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>•  The Dashboard totals foreign bank charges separately so your forex figure stays clean.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="20" customHeight="1">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>CONVENTIONS</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="15" customHeight="1">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>•  Rate = units of base currency per 1 unit of foreign currency (e.g. INR per 1 USD).</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="15" customHeight="1">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>•  Blue headers = your input.   Grey headers = automatically calculated, do not overtype.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="28" customHeight="1">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>•  Tables auto-extend: start typing on the row below a table and the formatting &amp; formulas copy down.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="28" customHeight="1">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
           <t>•  Dropdowns are provided for Type and Currency; Invoice No / Settlement Ref pick-lists are validated.</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="28" customHeight="1">
-      <c r="A32" s="4" t="inlineStr">
+    <row r="39" ht="28" customHeight="1">
+      <c r="A39" s="4" t="inlineStr">
         <is>
           <t>•  The sample rows are a worked example covering every scenario above – clear them to start your own data.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="28">
+  <mergeCells count="34">
     <mergeCell ref="A9:H9"/>
     <mergeCell ref="A30:H30"/>
+    <mergeCell ref="A39:H39"/>
     <mergeCell ref="A15:H15"/>
     <mergeCell ref="A24:H24"/>
+    <mergeCell ref="A36:H36"/>
     <mergeCell ref="A11:H11"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A6:H6"/>
     <mergeCell ref="A7:H7"/>
     <mergeCell ref="A25:H25"/>
     <mergeCell ref="A16:H16"/>
+    <mergeCell ref="A37:H37"/>
     <mergeCell ref="A27:H27"/>
     <mergeCell ref="A12:H12"/>
     <mergeCell ref="A18:H18"/>
@@ -1009,11 +1062,14 @@
     <mergeCell ref="A22:H22"/>
     <mergeCell ref="A4:H4"/>
     <mergeCell ref="A29:H29"/>
+    <mergeCell ref="A35:H35"/>
     <mergeCell ref="A20:H20"/>
+    <mergeCell ref="A38:H38"/>
     <mergeCell ref="A28:H28"/>
     <mergeCell ref="A13:H13"/>
     <mergeCell ref="A19:H19"/>
     <mergeCell ref="A31:H31"/>
+    <mergeCell ref="A34:H34"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1762,21 +1818,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:P12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
     <col width="9" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="15" customWidth="1" min="11" max="11"/>
-    <col width="40" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="17" customWidth="1" min="9" max="9"/>
+    <col width="17" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="15" customWidth="1" min="15" max="15"/>
+    <col width="44" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -1789,7 +1849,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="28" t="inlineStr">
         <is>
-          <t>Every money movement in foreign currency — receipts settle sales, payments settle purchases, incl. advances</t>
+          <t>Every money movement in foreign currency — receipts settle sales, payments settle purchases, incl. advances &amp; bank charges</t>
         </is>
       </c>
     </row>
@@ -1821,7 +1881,7 @@
       </c>
       <c r="F4" s="15" t="inlineStr">
         <is>
-          <t>FC Amount</t>
+          <t>FC Amount (Gross)</t>
         </is>
       </c>
       <c r="G4" s="15" t="inlineStr">
@@ -1829,27 +1889,47 @@
           <t>Settlement Rate</t>
         </is>
       </c>
-      <c r="H4" s="21" t="inlineStr">
+      <c r="H4" s="22" t="inlineStr">
+        <is>
+          <t>Foreign Bank Charges (FC)</t>
+        </is>
+      </c>
+      <c r="I4" s="21" t="inlineStr">
+        <is>
+          <t>Net Bank Movement (FC)</t>
+        </is>
+      </c>
+      <c r="J4" s="21" t="inlineStr">
         <is>
           <t>Settlement Value (Base)</t>
         </is>
       </c>
-      <c r="I4" s="21" t="inlineStr">
+      <c r="K4" s="21" t="inlineStr">
+        <is>
+          <t>Bank Charges (Base)</t>
+        </is>
+      </c>
+      <c r="L4" s="21" t="inlineStr">
+        <is>
+          <t>Net Bank Movement (Base)</t>
+        </is>
+      </c>
+      <c r="M4" s="21" t="inlineStr">
         <is>
           <t>FC Allocated</t>
         </is>
       </c>
-      <c r="J4" s="21" t="inlineStr">
+      <c r="N4" s="21" t="inlineStr">
         <is>
           <t>FC Unallocated</t>
         </is>
       </c>
-      <c r="K4" s="21" t="inlineStr">
+      <c r="O4" s="21" t="inlineStr">
         <is>
           <t>Allocation Status</t>
         </is>
       </c>
-      <c r="L4" s="15" t="inlineStr">
+      <c r="P4" s="15" t="inlineStr">
         <is>
           <t>Narration</t>
         </is>
@@ -1885,23 +1965,38 @@
       <c r="G5" s="17" t="n">
         <v>81.5</v>
       </c>
-      <c r="H5" s="24">
-        <f>[@[FC Amount]]*[@[Settlement Rate]]</f>
-        <v/>
+      <c r="H5" s="24" t="n">
+        <v>0</v>
       </c>
       <c r="I5" s="24">
+        <f>IF([@[Settlement Type]]="Receipt",[@[FC Amount (Gross)]]-[@[Foreign Bank Charges (FC)]],[@[FC Amount (Gross)]]+[@[Foreign Bank Charges (FC)]])</f>
+        <v/>
+      </c>
+      <c r="J5" s="24">
+        <f>[@[FC Amount (Gross)]]*[@[Settlement Rate]]</f>
+        <v/>
+      </c>
+      <c r="K5" s="24">
+        <f>[@[Foreign Bank Charges (FC)]]*[@[Settlement Rate]]</f>
+        <v/>
+      </c>
+      <c r="L5" s="24">
+        <f>[@[Net Bank Movement (FC)]]*[@[Settlement Rate]]</f>
+        <v/>
+      </c>
+      <c r="M5" s="24">
         <f>SUMIFS(tblAllocations[FC Allocated],tblAllocations[Settlement Ref],[@[Settlement Ref]])</f>
         <v/>
       </c>
-      <c r="J5" s="24">
-        <f>[@[FC Amount]]-[@[FC Allocated]]</f>
-        <v/>
-      </c>
-      <c r="K5" s="25">
+      <c r="N5" s="24">
+        <f>[@[FC Amount (Gross)]]-[@[FC Allocated]]</f>
+        <v/>
+      </c>
+      <c r="O5" s="25">
         <f>IF(ROUND([@[FC Unallocated]],2)=0,"Fully Allocated",IF([@[FC Allocated]]=0,"Unallocated","Partly Allocated"))</f>
         <v/>
       </c>
-      <c r="L5" s="16" t="inlineStr">
+      <c r="P5" s="16" t="inlineStr">
         <is>
           <t>Part advance received before invoice INV-S-001</t>
         </is>
@@ -1937,25 +2032,40 @@
       <c r="G6" s="17" t="n">
         <v>83</v>
       </c>
-      <c r="H6" s="24">
-        <f>[@[FC Amount]]*[@[Settlement Rate]]</f>
-        <v/>
+      <c r="H6" s="24" t="n">
+        <v>20</v>
       </c>
       <c r="I6" s="24">
+        <f>IF([@[Settlement Type]]="Receipt",[@[FC Amount (Gross)]]-[@[Foreign Bank Charges (FC)]],[@[FC Amount (Gross)]]+[@[Foreign Bank Charges (FC)]])</f>
+        <v/>
+      </c>
+      <c r="J6" s="24">
+        <f>[@[FC Amount (Gross)]]*[@[Settlement Rate]]</f>
+        <v/>
+      </c>
+      <c r="K6" s="24">
+        <f>[@[Foreign Bank Charges (FC)]]*[@[Settlement Rate]]</f>
+        <v/>
+      </c>
+      <c r="L6" s="24">
+        <f>[@[Net Bank Movement (FC)]]*[@[Settlement Rate]]</f>
+        <v/>
+      </c>
+      <c r="M6" s="24">
         <f>SUMIFS(tblAllocations[FC Allocated],tblAllocations[Settlement Ref],[@[Settlement Ref]])</f>
         <v/>
       </c>
-      <c r="J6" s="24">
-        <f>[@[FC Amount]]-[@[FC Allocated]]</f>
-        <v/>
-      </c>
-      <c r="K6" s="25">
+      <c r="N6" s="24">
+        <f>[@[FC Amount (Gross)]]-[@[FC Allocated]]</f>
+        <v/>
+      </c>
+      <c r="O6" s="25">
         <f>IF(ROUND([@[FC Unallocated]],2)=0,"Fully Allocated",IF([@[FC Allocated]]=0,"Unallocated","Partly Allocated"))</f>
         <v/>
       </c>
-      <c r="L6" s="16" t="inlineStr">
-        <is>
-          <t>2nd receipt against INV-S-001</t>
+      <c r="P6" s="16" t="inlineStr">
+        <is>
+          <t>2nd receipt against INV-S-001 (bank charge USD 20 deducted)</t>
         </is>
       </c>
     </row>
@@ -1989,23 +2099,38 @@
       <c r="G7" s="17" t="n">
         <v>83.40000000000001</v>
       </c>
-      <c r="H7" s="24">
-        <f>[@[FC Amount]]*[@[Settlement Rate]]</f>
-        <v/>
+      <c r="H7" s="24" t="n">
+        <v>0</v>
       </c>
       <c r="I7" s="24">
+        <f>IF([@[Settlement Type]]="Receipt",[@[FC Amount (Gross)]]-[@[Foreign Bank Charges (FC)]],[@[FC Amount (Gross)]]+[@[Foreign Bank Charges (FC)]])</f>
+        <v/>
+      </c>
+      <c r="J7" s="24">
+        <f>[@[FC Amount (Gross)]]*[@[Settlement Rate]]</f>
+        <v/>
+      </c>
+      <c r="K7" s="24">
+        <f>[@[Foreign Bank Charges (FC)]]*[@[Settlement Rate]]</f>
+        <v/>
+      </c>
+      <c r="L7" s="24">
+        <f>[@[Net Bank Movement (FC)]]*[@[Settlement Rate]]</f>
+        <v/>
+      </c>
+      <c r="M7" s="24">
         <f>SUMIFS(tblAllocations[FC Allocated],tblAllocations[Settlement Ref],[@[Settlement Ref]])</f>
         <v/>
       </c>
-      <c r="J7" s="24">
-        <f>[@[FC Amount]]-[@[FC Allocated]]</f>
-        <v/>
-      </c>
-      <c r="K7" s="25">
+      <c r="N7" s="24">
+        <f>[@[FC Amount (Gross)]]-[@[FC Allocated]]</f>
+        <v/>
+      </c>
+      <c r="O7" s="25">
         <f>IF(ROUND([@[FC Unallocated]],2)=0,"Fully Allocated",IF([@[FC Allocated]]=0,"Unallocated","Partly Allocated"))</f>
         <v/>
       </c>
-      <c r="L7" s="16" t="inlineStr">
+      <c r="P7" s="16" t="inlineStr">
         <is>
           <t>Final receipt against INV-S-001 (settled over 3 dates)</t>
         </is>
@@ -2041,25 +2166,40 @@
       <c r="G8" s="17" t="n">
         <v>83</v>
       </c>
-      <c r="H8" s="24">
-        <f>[@[FC Amount]]*[@[Settlement Rate]]</f>
-        <v/>
+      <c r="H8" s="24" t="n">
+        <v>100</v>
       </c>
       <c r="I8" s="24">
+        <f>IF([@[Settlement Type]]="Receipt",[@[FC Amount (Gross)]]-[@[Foreign Bank Charges (FC)]],[@[FC Amount (Gross)]]+[@[Foreign Bank Charges (FC)]])</f>
+        <v/>
+      </c>
+      <c r="J8" s="24">
+        <f>[@[FC Amount (Gross)]]*[@[Settlement Rate]]</f>
+        <v/>
+      </c>
+      <c r="K8" s="24">
+        <f>[@[Foreign Bank Charges (FC)]]*[@[Settlement Rate]]</f>
+        <v/>
+      </c>
+      <c r="L8" s="24">
+        <f>[@[Net Bank Movement (FC)]]*[@[Settlement Rate]]</f>
+        <v/>
+      </c>
+      <c r="M8" s="24">
         <f>SUMIFS(tblAllocations[FC Allocated],tblAllocations[Settlement Ref],[@[Settlement Ref]])</f>
         <v/>
       </c>
-      <c r="J8" s="24">
-        <f>[@[FC Amount]]-[@[FC Allocated]]</f>
-        <v/>
-      </c>
-      <c r="K8" s="25">
+      <c r="N8" s="24">
+        <f>[@[FC Amount (Gross)]]-[@[FC Allocated]]</f>
+        <v/>
+      </c>
+      <c r="O8" s="25">
         <f>IF(ROUND([@[FC Unallocated]],2)=0,"Fully Allocated",IF([@[FC Allocated]]=0,"Unallocated","Partly Allocated"))</f>
         <v/>
       </c>
-      <c r="L8" s="16" t="inlineStr">
-        <is>
-          <t>Single receipt settling two invoices INV-S-002 &amp; INV-S-003</t>
+      <c r="P8" s="16" t="inlineStr">
+        <is>
+          <t>Party transferred USD 20,000; bank deducted USD 100 foreign charges; net received USD 19,900. Settles INV-S-002 &amp; INV-S-003</t>
         </is>
       </c>
     </row>
@@ -2093,23 +2233,38 @@
       <c r="G9" s="17" t="n">
         <v>104.5</v>
       </c>
-      <c r="H9" s="24">
-        <f>[@[FC Amount]]*[@[Settlement Rate]]</f>
-        <v/>
+      <c r="H9" s="24" t="n">
+        <v>15</v>
       </c>
       <c r="I9" s="24">
+        <f>IF([@[Settlement Type]]="Receipt",[@[FC Amount (Gross)]]-[@[Foreign Bank Charges (FC)]],[@[FC Amount (Gross)]]+[@[Foreign Bank Charges (FC)]])</f>
+        <v/>
+      </c>
+      <c r="J9" s="24">
+        <f>[@[FC Amount (Gross)]]*[@[Settlement Rate]]</f>
+        <v/>
+      </c>
+      <c r="K9" s="24">
+        <f>[@[Foreign Bank Charges (FC)]]*[@[Settlement Rate]]</f>
+        <v/>
+      </c>
+      <c r="L9" s="24">
+        <f>[@[Net Bank Movement (FC)]]*[@[Settlement Rate]]</f>
+        <v/>
+      </c>
+      <c r="M9" s="24">
         <f>SUMIFS(tblAllocations[FC Allocated],tblAllocations[Settlement Ref],[@[Settlement Ref]])</f>
         <v/>
       </c>
-      <c r="J9" s="24">
-        <f>[@[FC Amount]]-[@[FC Allocated]]</f>
-        <v/>
-      </c>
-      <c r="K9" s="25">
+      <c r="N9" s="24">
+        <f>[@[FC Amount (Gross)]]-[@[FC Allocated]]</f>
+        <v/>
+      </c>
+      <c r="O9" s="25">
         <f>IF(ROUND([@[FC Unallocated]],2)=0,"Fully Allocated",IF([@[FC Allocated]]=0,"Unallocated","Partly Allocated"))</f>
         <v/>
       </c>
-      <c r="L9" s="16" t="inlineStr">
+      <c r="P9" s="16" t="inlineStr">
         <is>
           <t>Part receipt against INV-S-004 (balance stays open)</t>
         </is>
@@ -2145,23 +2300,38 @@
       <c r="G10" s="17" t="n">
         <v>89.5</v>
       </c>
-      <c r="H10" s="24">
-        <f>[@[FC Amount]]*[@[Settlement Rate]]</f>
-        <v/>
+      <c r="H10" s="24" t="n">
+        <v>0</v>
       </c>
       <c r="I10" s="24">
+        <f>IF([@[Settlement Type]]="Receipt",[@[FC Amount (Gross)]]-[@[Foreign Bank Charges (FC)]],[@[FC Amount (Gross)]]+[@[Foreign Bank Charges (FC)]])</f>
+        <v/>
+      </c>
+      <c r="J10" s="24">
+        <f>[@[FC Amount (Gross)]]*[@[Settlement Rate]]</f>
+        <v/>
+      </c>
+      <c r="K10" s="24">
+        <f>[@[Foreign Bank Charges (FC)]]*[@[Settlement Rate]]</f>
+        <v/>
+      </c>
+      <c r="L10" s="24">
+        <f>[@[Net Bank Movement (FC)]]*[@[Settlement Rate]]</f>
+        <v/>
+      </c>
+      <c r="M10" s="24">
         <f>SUMIFS(tblAllocations[FC Allocated],tblAllocations[Settlement Ref],[@[Settlement Ref]])</f>
         <v/>
       </c>
-      <c r="J10" s="24">
-        <f>[@[FC Amount]]-[@[FC Allocated]]</f>
-        <v/>
-      </c>
-      <c r="K10" s="25">
+      <c r="N10" s="24">
+        <f>[@[FC Amount (Gross)]]-[@[FC Allocated]]</f>
+        <v/>
+      </c>
+      <c r="O10" s="25">
         <f>IF(ROUND([@[FC Unallocated]],2)=0,"Fully Allocated",IF([@[FC Allocated]]=0,"Unallocated","Partly Allocated"))</f>
         <v/>
       </c>
-      <c r="L10" s="16" t="inlineStr">
+      <c r="P10" s="16" t="inlineStr">
         <is>
           <t>Part payment against INV-P-001</t>
         </is>
@@ -2197,25 +2367,40 @@
       <c r="G11" s="17" t="n">
         <v>90.5</v>
       </c>
-      <c r="H11" s="24">
-        <f>[@[FC Amount]]*[@[Settlement Rate]]</f>
-        <v/>
+      <c r="H11" s="24" t="n">
+        <v>40</v>
       </c>
       <c r="I11" s="24">
+        <f>IF([@[Settlement Type]]="Receipt",[@[FC Amount (Gross)]]-[@[Foreign Bank Charges (FC)]],[@[FC Amount (Gross)]]+[@[Foreign Bank Charges (FC)]])</f>
+        <v/>
+      </c>
+      <c r="J11" s="24">
+        <f>[@[FC Amount (Gross)]]*[@[Settlement Rate]]</f>
+        <v/>
+      </c>
+      <c r="K11" s="24">
+        <f>[@[Foreign Bank Charges (FC)]]*[@[Settlement Rate]]</f>
+        <v/>
+      </c>
+      <c r="L11" s="24">
+        <f>[@[Net Bank Movement (FC)]]*[@[Settlement Rate]]</f>
+        <v/>
+      </c>
+      <c r="M11" s="24">
         <f>SUMIFS(tblAllocations[FC Allocated],tblAllocations[Settlement Ref],[@[Settlement Ref]])</f>
         <v/>
       </c>
-      <c r="J11" s="24">
-        <f>[@[FC Amount]]-[@[FC Allocated]]</f>
-        <v/>
-      </c>
-      <c r="K11" s="25">
+      <c r="N11" s="24">
+        <f>[@[FC Amount (Gross)]]-[@[FC Allocated]]</f>
+        <v/>
+      </c>
+      <c r="O11" s="25">
         <f>IF(ROUND([@[FC Unallocated]],2)=0,"Fully Allocated",IF([@[FC Allocated]]=0,"Unallocated","Partly Allocated"))</f>
         <v/>
       </c>
-      <c r="L11" s="16" t="inlineStr">
-        <is>
-          <t>Balance payment against INV-P-001 (settled over 2 dates)</t>
+      <c r="P11" s="16" t="inlineStr">
+        <is>
+          <t>Balance payment against INV-P-001; bank charged USD 40 extra (settled over 2 dates)</t>
         </is>
       </c>
     </row>
@@ -2249,23 +2434,38 @@
       <c r="G12" s="17" t="n">
         <v>88.5</v>
       </c>
-      <c r="H12" s="24">
-        <f>[@[FC Amount]]*[@[Settlement Rate]]</f>
-        <v/>
+      <c r="H12" s="24" t="n">
+        <v>0</v>
       </c>
       <c r="I12" s="24">
+        <f>IF([@[Settlement Type]]="Receipt",[@[FC Amount (Gross)]]-[@[Foreign Bank Charges (FC)]],[@[FC Amount (Gross)]]+[@[Foreign Bank Charges (FC)]])</f>
+        <v/>
+      </c>
+      <c r="J12" s="24">
+        <f>[@[FC Amount (Gross)]]*[@[Settlement Rate]]</f>
+        <v/>
+      </c>
+      <c r="K12" s="24">
+        <f>[@[Foreign Bank Charges (FC)]]*[@[Settlement Rate]]</f>
+        <v/>
+      </c>
+      <c r="L12" s="24">
+        <f>[@[Net Bank Movement (FC)]]*[@[Settlement Rate]]</f>
+        <v/>
+      </c>
+      <c r="M12" s="24">
         <f>SUMIFS(tblAllocations[FC Allocated],tblAllocations[Settlement Ref],[@[Settlement Ref]])</f>
         <v/>
       </c>
-      <c r="J12" s="24">
-        <f>[@[FC Amount]]-[@[FC Allocated]]</f>
-        <v/>
-      </c>
-      <c r="K12" s="25">
+      <c r="N12" s="24">
+        <f>[@[FC Amount (Gross)]]-[@[FC Allocated]]</f>
+        <v/>
+      </c>
+      <c r="O12" s="25">
         <f>IF(ROUND([@[FC Unallocated]],2)=0,"Fully Allocated",IF([@[FC Allocated]]=0,"Unallocated","Partly Allocated"))</f>
         <v/>
       </c>
-      <c r="L12" s="16" t="inlineStr">
+      <c r="P12" s="16" t="inlineStr">
         <is>
           <t>Advance paid before invoice INV-P-002</t>
         </is>
@@ -2273,8 +2473,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:L2"/>
-    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A1:P1"/>
+    <mergeCell ref="A2:P2"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation sqref="B5:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
@@ -3235,7 +3435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -3392,90 +3592,147 @@
     </row>
     <row r="18"/>
     <row r="19" ht="20" customHeight="1">
-      <c r="B19" s="7" t="inlineStr">
-        <is>
-          <t>DATA OVERVIEW</t>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>FOREIGN BANK CHARGES  (separate expense — not forex)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="30" t="inlineStr">
         <is>
-          <t>Invoices captured</t>
+          <t>Total Foreign Bank Charges (FC)</t>
         </is>
       </c>
       <c r="C20" s="12" t="n"/>
       <c r="D20" s="32">
-        <f>COUNTA(tblInvoices[Invoice No])</f>
+        <f>SUM(tblSettlements[Foreign Bank Charges (FC)])</f>
         <v/>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="30" t="inlineStr">
         <is>
-          <t>Receipts &amp; Payments captured</t>
+          <t>Total Foreign Bank Charges (Base)</t>
         </is>
       </c>
       <c r="C21" s="12" t="n"/>
       <c r="D21" s="32">
-        <f>COUNTA(tblSettlements[Settlement Ref])</f>
+        <f>SUM(tblSettlements[Bank Charges (Base)])</f>
         <v/>
       </c>
     </row>
     <row r="22">
       <c r="B22" s="30" t="inlineStr">
         <is>
-          <t>Allocation lines</t>
+          <t>Net Cash Received — receipts (Base)</t>
         </is>
       </c>
       <c r="C22" s="12" t="n"/>
       <c r="D22" s="32">
-        <f>COUNTA(tblAllocations[Alloc ID])</f>
+        <f>SUMIFS(tblSettlements[Net Bank Movement (Base)],tblSettlements[Settlement Type],"Receipt")</f>
         <v/>
       </c>
     </row>
     <row r="23">
       <c r="B23" s="30" t="inlineStr">
         <is>
-          <t>Advance settlements</t>
+          <t>Net Cash Paid — payments (Base)</t>
         </is>
       </c>
       <c r="C23" s="12" t="n"/>
       <c r="D23" s="32">
+        <f>SUMIFS(tblSettlements[Net Bank Movement (Base)],tblSettlements[Settlement Type],"Payment")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24"/>
+    <row r="25" ht="20" customHeight="1">
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>DATA OVERVIEW</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="30" t="inlineStr">
+        <is>
+          <t>Invoices captured</t>
+        </is>
+      </c>
+      <c r="C26" s="12" t="n"/>
+      <c r="D26" s="33">
+        <f>COUNTA(tblInvoices[Invoice No])</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="30" t="inlineStr">
+        <is>
+          <t>Receipts &amp; Payments captured</t>
+        </is>
+      </c>
+      <c r="C27" s="12" t="n"/>
+      <c r="D27" s="33">
+        <f>COUNTA(tblSettlements[Settlement Ref])</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="30" t="inlineStr">
+        <is>
+          <t>Allocation lines</t>
+        </is>
+      </c>
+      <c r="C28" s="12" t="n"/>
+      <c r="D28" s="33">
+        <f>COUNTA(tblAllocations[Alloc ID])</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="30" t="inlineStr">
+        <is>
+          <t>Advance settlements</t>
+        </is>
+      </c>
+      <c r="C29" s="12" t="n"/>
+      <c r="D29" s="33">
         <f>COUNTIF(tblAllocations[Settlement Nature],"Advance")</f>
         <v/>
       </c>
     </row>
-    <row r="24">
-      <c r="B24" s="30" t="inlineStr">
+    <row r="30">
+      <c r="B30" s="30" t="inlineStr">
         <is>
           <t>Invoices fully settled</t>
         </is>
       </c>
-      <c r="C24" s="12" t="n"/>
-      <c r="D24" s="32">
+      <c r="C30" s="12" t="n"/>
+      <c r="D30" s="33">
         <f>COUNTIF(tblInvoices[Settlement Status],"Fully Settled")</f>
         <v/>
       </c>
     </row>
-    <row r="25">
-      <c r="B25" s="30" t="inlineStr">
+    <row r="31">
+      <c r="B31" s="30" t="inlineStr">
         <is>
           <t>Invoices part/open</t>
         </is>
       </c>
-      <c r="C25" s="12" t="n"/>
-      <c r="D25" s="32">
+      <c r="C31" s="12" t="n"/>
+      <c r="D31" s="33">
         <f>COUNTIFS(tblInvoices[Settlement Status],"&lt;&gt;Fully Settled")</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="21">
+  <mergeCells count="26">
     <mergeCell ref="B11:D11"/>
     <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B25:C25"/>
     <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B27:C27"/>
     <mergeCell ref="B12:C12"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="B21:C21"/>
@@ -3485,14 +3742,18 @@
     <mergeCell ref="B17:C17"/>
     <mergeCell ref="B8:C8"/>
     <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B29:C29"/>
     <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B28:C28"/>
     <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B25:D25"/>
     <mergeCell ref="B16:D16"/>
     <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B30:C30"/>
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B26:C26"/>
   </mergeCells>
   <conditionalFormatting sqref="D5">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">

</xml_diff>